<commit_message>
feat: update Helios PRD automation, launcher and tests
</commit_message>
<xml_diff>
--- a/data/Helios_Material_Lines_Template.xlsx
+++ b/data/Helios_Material_Lines_Template.xlsx
@@ -1,15 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Material Lines Entry" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Material Lines Entry" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Material Lines Entry'!$A$1:$E$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,12 +32,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="0064748B"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -78,13 +74,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -162,6 +155,41 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Helios PRD</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Part code in catalog (e.g. CABL00058)</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Positive number (e.g. 1)</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Site identifier (e.g. TZKA8027)</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Cost Code - SAP Budget Line (e.g. 2026_2.2.1.)</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>WBS and Project Code (e.g. TZKA8027-1795051262)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -453,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -491,362 +519,694 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Format: Part code in catalog (e.g. CABL00058)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Format: Positive number (e.g. 1)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Format: Site identifier (e.g. TZKA8027)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Format: Cost Code - SAP Budget Line (e.g. 2026_2.2.1.)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Format: WBS and Project Code (e.g. TZKA8027-1795051262)</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n"/>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n"/>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n"/>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n"/>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="3" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n"/>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n"/>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n"/>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="3" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n"/>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n"/>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n"/>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="3" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n"/>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="3" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n"/>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="3" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n"/>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="3" t="n"/>
-      <c r="D47" s="3" t="n"/>
-      <c r="E47" s="3" t="n"/>
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="3" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n"/>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="3" t="n"/>
-      <c r="D48" s="3" t="n"/>
-      <c r="E48" s="3" t="n"/>
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="3" t="n"/>
-      <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="3" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="3" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="3" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="3" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="3" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="3" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="3" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="3" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="3" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="3" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="3" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="3" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="3" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="3" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="3" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="3" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="3" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="3" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="3" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="3" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="3" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="3" t="n"/>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n"/>
+      <c r="B73" s="3" t="n"/>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" s="2" t="n"/>
+      <c r="E73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n"/>
+      <c r="B74" s="3" t="n"/>
+      <c r="C74" s="2" t="n"/>
+      <c r="D74" s="2" t="n"/>
+      <c r="E74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="3" t="n"/>
+      <c r="C75" s="2" t="n"/>
+      <c r="D75" s="2" t="n"/>
+      <c r="E75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n"/>
+      <c r="B76" s="3" t="n"/>
+      <c r="C76" s="2" t="n"/>
+      <c r="D76" s="2" t="n"/>
+      <c r="E76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="3" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n"/>
+      <c r="B78" s="3" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="3" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
+      <c r="E79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n"/>
+      <c r="B80" s="3" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+      <c r="E80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n"/>
+      <c r="B81" s="3" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="2" t="n"/>
+      <c r="E81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="3" t="n"/>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" s="2" t="n"/>
+      <c r="E82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n"/>
+      <c r="B83" s="3" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
+      <c r="E83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="3" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n"/>
+      <c r="E84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="3" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="3" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+      <c r="E86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="3" t="n"/>
+      <c r="C87" s="2" t="n"/>
+      <c r="D87" s="2" t="n"/>
+      <c r="E87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="3" t="n"/>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
+      <c r="E88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="3" t="n"/>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
+      <c r="E89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="3" t="n"/>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" s="2" t="n"/>
+      <c r="E90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="3" t="n"/>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" s="2" t="n"/>
+      <c r="E91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="3" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
+      <c r="E92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n"/>
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n"/>
+      <c r="E93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="2" t="n"/>
+      <c r="E94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n"/>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="2" t="n"/>
+      <c r="D95" s="2" t="n"/>
+      <c r="E95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+      <c r="B96" s="3" t="n"/>
+      <c r="C96" s="2" t="n"/>
+      <c r="D96" s="2" t="n"/>
+      <c r="E96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="2" t="n"/>
+      <c r="D97" s="2" t="n"/>
+      <c r="E97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="3" t="n"/>
+      <c r="C98" s="2" t="n"/>
+      <c r="D98" s="2" t="n"/>
+      <c r="E98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n"/>
+      <c r="B99" s="3" t="n"/>
+      <c r="C99" s="2" t="n"/>
+      <c r="D99" s="2" t="n"/>
+      <c r="E99" s="2" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>